<commit_message>
Tok fází soutěže: pole entry + phase_order do SYSTEM + feeds_into/loser
Model fází jedné soutěže (ZČ → play-off / o záchranu, poražení ČF → sk. 5-8…):
- harmonize_schema: do SYSTEM přidána pole 'entry' (kdo do fáze vstupuje) a
  'phase_order' (pořadí fáze); feeds_into = vítězná větev, feeds_into_loser = poražení
- phase_flow.py: deklarativní populátor (scope L10 + jednoznačný název) + read-only
  report toku; vzorově vyplněno 1988/89 (přesně ZČ→ČF→SF→F, ČF→O5-8, 9-12→o udržení)
  a 2013/14 (předkolo 7-10, play out 11-14)
- build_db: competitions.entry + competitions.phase_order protékají do almanach.sqlite
- docs/CLAUDE_FAZE_SOUTEZI.md §3.6: konvence kódování toku fází
- README aktualizován

Ostatní sezóny mají pole prázdná — populace dalších = postupně (každý formát zvlášť).
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -1625,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1687,6 +1687,16 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>prev_node_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>phase_order</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plošně vyplnit tok fází všech soutěží (phase_flow.py --auto): 633 soutěží
Automatická inference toku fází ze struktury (názvy uzlů + competition_type +
seskupení po soutěžích přes parent_node_id + počty týmů z tabulek pro pozice):
- entry, phase_order, feeds_into, feeds_into_loser vyplněno pro 2200 uzlů fází
  v 73 ze 74 sezón (633 soutěží — extraliga i nižší/krajské playoffy nezávisle)
- ZČ → play-off (horní) / o udržení (dolní); ČF → SF / O 5.-8.; SF → finále / O 3.;
  předkolo, play out, osmifinále atd.; pozice 1.–8./9.–12. počítány z velikostí tabulek
- feeds_into 595→1409 (baráž/kvalifikace zachovány, přidán vnitřní tok)
- build_db: entry+phase_order protékají do almanach.sqlite
- docs/CLAUDE_FAZE_SOUTEZI.md + README aktualizovány

Heuristika — u exotických formátů může být entry/tok přibližný, lze přepsat ručně.
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -1837,6 +1837,8 @@
           <t>NODE_S1947_48_0001</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -1846,6 +1848,14 @@
         <is>
           <t>LTC Praha – I. ČLTK Praha 7:1, 13:5</t>
         </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>vítězové SF</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1947/48: doplnit vše ostatní z PDF (Mistrovství Slovenska + poznámky)
enrich_1947_48.py (in-place, zachová TODO i pole fází):
- Mistrovství Slovenska (Poprad 28.-29.2.1948) jako reálná tabulka — list 30SVK
  + SYSTEM uzel + CLUBS (Tatry Poprad mistr, Trenčín, Kežmarok; Spišská N.V. vyloučena).
  Ověřeno: suma GF=GA 51:51, body sedí.
- NOTES: anulace divize/žup (počasí 13.2.1948), Středočeský divizní pohár (náhradní
  vyřazovák), nedohraná kvalifikace + přechod na 8člennou ligu 1948/49 (ATK přidán,
  Podolí zaniklo), postup do MS divize (Těšetice-Ostravská Slavia), slovenský
  titulový zápas ŠK Bratislava-VŠ Bratislava 4:3, sloučení Pokojovice+Okříšky.
- META: mistr_slovenska Tatry Poprad, status PARTIAL (divize anulovány).
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -14,6 +14,7 @@
     <sheet name="META" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="NOTES" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="TODO" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="30SVK" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TODO'!$A$1:$F$2</definedName>
@@ -1625,7 +1626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1837,8 +1838,6 @@
           <t>NODE_S1947_48_0001</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -1857,6 +1856,50 @@
       <c r="N5" t="n">
         <v>5</v>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>regional_championship</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>REG_SVK</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2-1-0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>28.–29. 2. 1948, Poprad. AC Spišská Nová Ves vyloučena.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1869,7 +1912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2370,6 +2413,166 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>Havlíčkův Brod</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HC Tatry Poprad</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>HC Tatry Poprad [M-SVK]</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>30SVK</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Poprad</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TTS Trenčín</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TTS Trenčín</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>30SVK</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Trenčín</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ŠK Kežmarok</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ŠK Kežmarok</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>30SVK</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Kežmarok</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AC Spišská Nová Ves</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AC Spišská Nová Ves</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska — vyloučena ze soutěže (bez záznamu v tabulce).</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Spišská Nová Ves</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2467,7 +2670,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2682,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2694,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PARTIAL — pouze nejvyšší soutěž (Státní liga). Nižší a regiony zatím nezpracovány.</t>
+          <t>PARTIAL — Státní liga + Mistrovství Slovenska (tabulky). Divize a župní soutěže anulovány (počasí) — jen poznámky.</t>
         </is>
       </c>
     </row>
@@ -2528,6 +2731,18 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>Navázáno dopředu na S1948_49 (prev_club_id doplněn tam u doložených klubů). Prev na S1946_47 zatím prázdný.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mistr_slovenska</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HC Tatry Poprad</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2584,6 +2799,83 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>Nižší a krajské soutěže 1947/48 ZATÍM NEZPRACOVÁNY — přijdou později (chirurgicky).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nižší soutěže (divize i župní) byly 13. 2. 1948 Českým svazem prohlášeny za nesehrané a ANULOVÁNY pro nepřízeň počasí (zimní stadiony odmítly finanční riziko).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Výjimka: mistři župy slezské a hanácké směli sehrát zápas o 6. účastníka skupiny A Moravskoslezské divize.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska (28.–29. 2. 1948, Poprad): 1. HC Tatry Poprad, 2. TTS Trenčín, 3. ŠK Kežmarok; AC Spišská Nová Ves vyloučena ze soutěže.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Středočeská divizní soutěž nahrazena vyřazovacím turnajem (Středočeský divizní pohár) na ZS Štvanice (1. kolo, čtvrtfinále, semifinále). Finále se nehrálo (mělo být až příští sezónu Slavia–Starokolínský, ale nestalo se); výsledek 2. semifinále není doložen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kvalifikace o Státní ligu (turnaj divizních vítězů) se pro počasí nedohrála.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Přechod na jednoskupinovou Státní ligu o 8 účastnících: poslední 2 z každé skupiny sestoupily; bez kvalifikace zařazen nově vzniklý ATK Praha (→ 9 týmů), pak HC Stadion Podolí ukončil činnost → 1948/49 hrálo 8 klubů.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>O postup do Moravskoslezské divize: SK Těšetice – SK Ostravská Slavia 1:15; odveta nehrána (Těšetice vzdaly) → postoupila SK Ostravská Slavia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Po sezóně sloučení HC Viktoria HPH Pokojovice s SK Okříšky.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Východoslovenská župa — jediný doložený výsledek: AC Veľký Šariš – ŠK Slávia Prešov 2:9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Neoficiální mistr Slovenska (zápas dvou bratislavských klubů ze Státní ligy): ŠK Bratislava – VŠ Bratislava 4:3 (11. 12. 1947).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Původní (nesehrané) rozlosování všech divizí je v podkladech doloženo včetně soupisek skupin.</t>
         </is>
       </c>
     </row>
@@ -2652,4 +2944,424 @@
   <autoFilter ref="A1:F2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>row_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>block_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>club_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>GF</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>comp_path</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>club_id</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>prev_club_id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>dest_node_id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>dest_type</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>season_fate</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>tr_id</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0005</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>HC Tatry Poprad</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>37</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0005</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0013</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TR_S1947_48_10001</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TTS Trenčín</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>18</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0005</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0014</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TR_S1947_48_10002</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ŠK Kežmarok</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>:</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>31</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Mistrovství Slovenska</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0005</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>L30</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>CLUB_S1947_48_0015</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TR_S1947_48_10003</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Konsolidace: refresh odvozených dat po všech úpravách (TODO/fáze/prev_node_id/DB)
Idempotentní refresh napříč 74 sezónami po champion+divize+oblastní opravách:
harmonize_schema, add_prev_node_id, phase_flow --auto, apply_todo_sheets, build_db,
validate_almanach, health. Integrita čistá: 0 rozbitých chainů, 0 nekonzistencí
fate, 0 orphanů; app načítá 74 sezón.
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -13,11 +13,11 @@
     <sheet name="CLUBS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="META" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="NOTES" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TODO" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="30SVK" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="30SVK" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TODO" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TODO'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TODO'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1883,23 +1883,16 @@
           <t>REG_SVK</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>2-1-0</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>28.–29. 2. 1948, Poprad. AC Spišská Nová Ves vyloučena.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2447,8 +2440,6 @@
           <t>L30</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
@@ -2481,14 +2472,11 @@
           <t>30SVK</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>L30</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
@@ -2521,14 +2509,11 @@
           <t>30SVK</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>L30</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>Mistrovství Slovenska (Poprad). prev_club_id zatím prázdný.</t>
@@ -2556,15 +2541,11 @@
           <t>AC Spišská Nová Ves</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>L30</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>Mistrovství Slovenska — vyloučena ze soutěže (bez záznamu v tabulce).</t>
@@ -2885,68 +2866,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="88" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>typ</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>popis</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>vyřešeno? (ANO/ne)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>poznámka kolegy</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>(žádné otevřené položky — sezóna OK)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3108,18 +3027,6 @@
           <t>Mistrovství Slovenska</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
           <t>NODE_S1947_48_0005</t>
@@ -3130,13 +3037,6 @@
           <t>L30</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3144,7 +3044,6 @@
           <t>T</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
         <v>1</v>
       </c>
@@ -3204,16 +3103,11 @@
           <t>CLUB_S1947_48_0013</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>TR_S1947_48_10001</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3221,7 +3115,6 @@
           <t>T</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>2</v>
       </c>
@@ -3230,7 +3123,6 @@
           <t>TTS Trenčín</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>2</v>
       </c>
@@ -3277,16 +3169,11 @@
           <t>CLUB_S1947_48_0014</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>TR_S1947_48_10002</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3294,7 +3181,6 @@
           <t>T</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
         <v>3</v>
       </c>
@@ -3303,7 +3189,6 @@
           <t>ŠK Kežmarok</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -3350,18 +3235,75 @@
           <t>CLUB_S1947_48_0015</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>TR_S1947_48_10003</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>typ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>popis</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>vyřešeno? (ANO/ne)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>poznámka kolegy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>(žádné otevřené položky — sezóna OK)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Torza: vloženy gapy do TODO listů základních xlsx (typ=torzo, oranžové, marker [torzo-audit])
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -41,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +53,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +68,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,11 +88,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -55512,11 +55523,30 @@
       </c>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>(žádné otevřené položky — sezóna OK)</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>torzo</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Podbrdská župa I. třída (Středočeský kraj) · NODE_S1947_48_0010</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>máme jen 2 týmy (SK Osov, Sparta Podluhy), chybí zbytek týmů a tabulka  [torzo-audit]</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F2"/>

</xml_diff>

<commit_message>
Torza do DB: re-runnable apply_torzo_gaps.py (TODO+NOTES), oprava plain NOTES 1947-49
</commit_message>
<xml_diff>
--- a/data/S1947_48_FINAL.xlsx
+++ b/data/S1947_48_FINAL.xlsx
@@ -88,13 +88,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -54965,13 +54968,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>note_text</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>node_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fake_club_ids</t>
         </is>
       </c>
     </row>
@@ -55084,6 +55107,23 @@
       <c r="A17" t="inlineStr">
         <is>
           <t>Původní (nesehrané) rozlosování všech divizí je v podkladech doloženo včetně soupisek skupin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[TBD] torzo: máme jen 2 týmy (SK Osov, Sparta Podluhy), chybí zbytek týmů a tabulka  [torzo-audit]</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NODE_S1947_48_0010</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TODO-auto</t>
         </is>
       </c>
     </row>
@@ -55536,7 +55576,7 @@
           <t>Podbrdská župa I. třída (Středočeský kraj) · NODE_S1947_48_0010</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>máme jen 2 týmy (SK Osov, Sparta Podluhy), chybí zbytek týmů a tabulka  [torzo-audit]</t>
         </is>

</xml_diff>